<commit_message>
lots to do in accessibility still
</commit_message>
<xml_diff>
--- a/data/static/output_graph/hazard_names.xlsx
+++ b/data/static/output_graph/hazard_names.xlsx
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>delfland_ghg200m_wgs84_processed</t>
+          <t>delfland_ghg200m_wgs84</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -468,14 +468,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>C:\python\powerpath\data\static\hazard\processed\delfland_ghg200m_wgs84_processed.tif</t>
+          <t>C:\python\powerpath\data\static\hazard\delfland_ghg200m_wgs84.tif</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>delfland_ghg200m_wgs84_processed</t>
+          <t>delfland_ghg200m_wgs84</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C:\python\powerpath\data\static\hazard\processed\delfland_ghg200m_wgs84_processed.tif</t>
+          <t>C:\python\powerpath\data\static\hazard\delfland_ghg200m_wgs84.tif</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recovery with access real flood data
Some issue persists stopping repairs from fully proceeding in the islands crew assignment method
</commit_message>
<xml_diff>
--- a/data/static/output_graph/hazard_names.xlsx
+++ b/data/static/output_graph/hazard_names.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-03_scale_5_wgs84.tif</t>
+          <t>N:\Projects\11209000\11209175\B. Measurements and calculations\Data\timeseries_data\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-03_scale_5_wgs84.tif</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-03_scale_5_wgs84.tif</t>
+          <t>N:\Projects\11209000\11209175\B. Measurements and calculations\Data\timeseries_data\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-03_scale_5_wgs84.tif</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-04_scale_5_wgs84.tif</t>
+          <t>N:\Projects\11209000\11209175\B. Measurements and calculations\Data\timeseries_data\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-04_scale_5_wgs84.tif</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-04_scale_5_wgs84.tif</t>
+          <t>N:\Projects\11209000\11209175\B. Measurements and calculations\Data\timeseries_data\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-04_scale_5_wgs84.tif</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-05_scale_5_wgs84.tif</t>
+          <t>N:\Projects\11209000\11209175\B. Measurements and calculations\Data\timeseries_data\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-05_scale_5_wgs84.tif</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-05_scale_5_wgs84.tif</t>
+          <t>N:\Projects\11209000\11209175\B. Measurements and calculations\Data\timeseries_data\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-05_scale_5_wgs84.tif</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-06_scale_5_wgs84.tif</t>
+          <t>N:\Projects\11209000\11209175\B. Measurements and calculations\Data\timeseries_data\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-06_scale_5_wgs84.tif</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-06_scale_5_wgs84.tif</t>
+          <t>N:\Projects\11209000\11209175\B. Measurements and calculations\Data\timeseries_data\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-06_scale_5_wgs84.tif</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-07_scale_5_wgs84.tif</t>
+          <t>N:\Projects\11209000\11209175\B. Measurements and calculations\Data\timeseries_data\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-07_scale_5_wgs84.tif</t>
         </is>
       </c>
     </row>
@@ -666,183 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-07_scale_5_wgs84.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-08_scale_5_wgs84</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>maximum</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>EV6_ma</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-08_scale_5_wgs84.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-08_scale_5_wgs84</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>fraction of network segment impacted by hazard</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>EV6_fr</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-08_scale_5_wgs84.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-09_scale_5_wgs84</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>maximum</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>EV7_ma</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-09_scale_5_wgs84.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-09_scale_5_wgs84</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>fraction of network segment impacted by hazard</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>EV7_fr</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-09_scale_5_wgs84.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-10_scale_5_wgs84</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>maximum</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>EV8_ma</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-10_scale_5_wgs84.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-10_scale_5_wgs84</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>fraction of network segment impacted by hazard</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>EV8_fr</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-10_scale_5_wgs84.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-11_scale_5_wgs84</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>maximum</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>EV9_ma</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-11_scale_5_wgs84.tif</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-11_scale_5_wgs84</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>fraction of network segment impacted by hazard</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>EV9_fr</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>C:\python\Use_case_stedin\hazard_maps_time_series_waterbom\hazard_timeseries\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GLG_waterschijf_1900-07-11_scale_5_wgs84.tif</t>
+          <t>N:\Projects\11209000\11209175\B. Measurements and calculations\Data\timeseries_data\reprojected\20220610 JF  Limburgbui 200 mm 48h  voormalen 15 cm  GHG_waterschijf_1900-01-07_scale_5_wgs84.tif</t>
         </is>
       </c>
     </row>

</xml_diff>